<commit_message>
Ship the 71-bus microgrid files the paper used
</commit_message>
<xml_diff>
--- a/grids/mg71_S1_baseline.xlsx
+++ b/grids/mg71_S1_baseline.xlsx
@@ -728,13 +728,13 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>876250</v>
+        <v>1752500</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>1</v>
@@ -760,10 +760,10 @@
         <v>1</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>876250</v>
+        <v>1752500</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>1</v>
@@ -789,10 +789,10 @@
         <v>1</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>876250</v>
+        <v>1752500</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>1</v>
@@ -818,10 +818,10 @@
         <v>1</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>876250</v>
+        <v>1752500</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>1</v>
@@ -7552,10 +7552,10 @@
         <v>35</v>
       </c>
       <c r="D35" s="2" t="n">
-        <v>1.9990663917</v>
+        <v>0.4997264657</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.19990663917</v>
+        <v>0.4997264657</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -7593,10 +7593,10 @@
         <v>36</v>
       </c>
       <c r="D36" s="2" t="n">
-        <v>1.9990663917</v>
+        <v>0.4997264657</v>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.19990663917</v>
+        <v>0.4997264657</v>
       </c>
       <c r="F36" s="6" t="n">
         <v>0</v>
@@ -7803,10 +7803,10 @@
         <v>10</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>928750</v>
+        <v>1857500</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>575000</v>
@@ -7838,10 +7838,10 @@
         <v>10</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>928750</v>
+        <v>1857500</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>575000</v>
@@ -7873,10 +7873,10 @@
         <v>10</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>928750</v>
+        <v>1857500</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>575000</v>
@@ -7908,10 +7908,10 @@
         <v>10</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5</v>
+        <v>1.25</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>928750</v>
+        <v>1857500</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>575000</v>
@@ -14153,11 +14153,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="18"/>
   <cols>
-    <col width="14.85546875" bestFit="1" customWidth="1" style="21" min="2" max="2"/>
-    <col width="14.5703125" bestFit="1" customWidth="1" style="21" min="5" max="5"/>
+    <col width="14.85546875" bestFit="1" customWidth="1" style="21" min="2" max="4"/>
+    <col width="14.5703125" bestFit="1" customWidth="1" style="21" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="19" customFormat="1" customHeight="1" s="1">
@@ -14168,25 +14168,35 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Nominal Current</t>
+          <t>Z_p</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>I_p</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>P_p</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>V0 [pu]</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>V_base [V]</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>VM min [pu]</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>VM max [pu]</t>
         </is>
@@ -14199,16 +14209,22 @@
       <c r="B2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C2" s="5" t="n">
-        <v>1</v>
+      <c r="C2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E2" s="2" t="n">
+      <c r="G2" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14220,15 +14236,21 @@
         <v>0</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E3" s="2" t="n">
+      <c r="G3" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14239,16 +14261,22 @@
       <c r="B4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="5" t="n">
-        <v>1</v>
+      <c r="C4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="G4" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14260,15 +14288,21 @@
         <v>0</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="G5" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14280,15 +14314,21 @@
         <v>0</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="G6" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14300,15 +14340,21 @@
         <v>0</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="G7" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14320,15 +14366,21 @@
         <v>0</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="G8" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14340,15 +14392,21 @@
         <v>0</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="G9" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14360,15 +14418,21 @@
         <v>0</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="G10" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14380,15 +14444,21 @@
         <v>0</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="G11" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14400,15 +14470,21 @@
         <v>0</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="G12" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14420,15 +14496,21 @@
         <v>0</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E13" s="2" t="n">
+      <c r="G13" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14440,15 +14522,21 @@
         <v>0</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="G14" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14460,15 +14548,21 @@
         <v>0</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E15" s="2" t="n">
+      <c r="G15" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14480,15 +14574,21 @@
         <v>0</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="G16" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14500,15 +14600,21 @@
         <v>0</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E17" s="2" t="n">
+      <c r="G17" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14520,15 +14626,21 @@
         <v>0</v>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="G18" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14540,15 +14652,21 @@
         <v>0</v>
       </c>
       <c r="C19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E19" s="2" t="n">
+      <c r="G19" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14560,15 +14678,21 @@
         <v>0</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="G20" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14580,15 +14704,21 @@
         <v>0</v>
       </c>
       <c r="C21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E21" s="2" t="n">
+      <c r="G21" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14600,15 +14730,21 @@
         <v>0</v>
       </c>
       <c r="C22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="G22" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14620,15 +14756,21 @@
         <v>0</v>
       </c>
       <c r="C23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E23" s="2" t="n">
+      <c r="G23" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F23" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14640,15 +14782,21 @@
         <v>0</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="G24" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F24" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14660,15 +14808,21 @@
         <v>0</v>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E25" s="2" t="n">
+      <c r="G25" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F25" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14680,15 +14834,21 @@
         <v>0</v>
       </c>
       <c r="C26" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="G26" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14700,15 +14860,21 @@
         <v>0</v>
       </c>
       <c r="C27" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="G27" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14720,15 +14886,21 @@
         <v>0</v>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E28" s="2" t="n">
+      <c r="G28" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14740,15 +14912,21 @@
         <v>0</v>
       </c>
       <c r="C29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E29" s="2" t="n">
+      <c r="G29" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F29" s="2" t="n">
+      <c r="H29" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14760,15 +14938,21 @@
         <v>0</v>
       </c>
       <c r="C30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E30" s="2" t="n">
+      <c r="G30" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F30" s="2" t="n">
+      <c r="H30" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14780,15 +14964,21 @@
         <v>0</v>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E31" s="2" t="n">
+      <c r="G31" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F31" s="2" t="n">
+      <c r="H31" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14800,15 +14990,21 @@
         <v>0</v>
       </c>
       <c r="C32" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E32" s="2" t="n">
+      <c r="G32" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F32" s="2" t="n">
+      <c r="H32" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14820,15 +15016,21 @@
         <v>0</v>
       </c>
       <c r="C33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E33" s="2" t="n">
+      <c r="G33" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F33" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>
@@ -14840,15 +15042,21 @@
         <v>0</v>
       </c>
       <c r="C34" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="2" t="n">
         <v>20670</v>
       </c>
-      <c r="E34" s="2" t="n">
+      <c r="G34" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="F34" s="2" t="n">
+      <c r="H34" s="2" t="n">
         <v>1.05</v>
       </c>
     </row>

</xml_diff>